<commit_message>
Separate split predecessors from successor entities
</commit_message>
<xml_diff>
--- a/data/releases/v2.0/china_city_entity_master_V2.0.xlsx
+++ b/data/releases/v2.0/china_city_entity_master_V2.0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市总表" sheetId="1" r:id="R6849269ba1a643d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市总表" sheetId="1" r:id="R72f66fb9520143c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4018,7 +4018,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H86" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1996</x:v>
       </x:c>
       <x:c r="I86" s="12" t="str">
         <x:v>2026</x:v>
@@ -4030,7 +4030,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L86" s="14" t="str">
-        <x:v>1987-2026 泰州市</x:v>
+        <x:v>1987-1995 [not_established]; 1996-2026 泰州市</x:v>
       </x:c>
       <x:c r="M86" s="15" t="str">
         <x:v>0</x:v>
@@ -4061,7 +4061,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H87" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1996</x:v>
       </x:c>
       <x:c r="I87" s="12" t="str">
         <x:v>2026</x:v>
@@ -4073,7 +4073,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L87" s="14" t="str">
-        <x:v>1987-2026 宿迁市</x:v>
+        <x:v>1987-1995 [not_established]; 1996-2026 宿迁市</x:v>
       </x:c>
       <x:c r="M87" s="15" t="str">
         <x:v>0</x:v>
@@ -9221,7 +9221,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H207" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1988</x:v>
       </x:c>
       <x:c r="I207" s="12" t="str">
         <x:v>2026</x:v>
@@ -9233,10 +9233,10 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L207" s="14" t="str">
-        <x:v>1987-1987 惠阳地区; 1988-2026 惠州市</x:v>
+        <x:v>1987-1987 [not_established]; 1988-2026 惠州市</x:v>
       </x:c>
       <x:c r="M207" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N207" s="14" t="str"/>
       <x:c r="O207" s="14" t="str"/>
@@ -10253,7 +10253,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H231" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>2002</x:v>
       </x:c>
       <x:c r="I231" s="12" t="str">
         <x:v>2026</x:v>
@@ -10262,13 +10262,13 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="K231" s="2" t="str">
-        <x:v>event_crosschecked</x:v>
+        <x:v>wikipedia_verified</x:v>
       </x:c>
       <x:c r="L231" s="14" t="str">
-        <x:v>1987-2001 南宁地区; 2002-2026 崇左市</x:v>
+        <x:v>1987-2001 [not_established]; 2002-2026 崇左市</x:v>
       </x:c>
       <x:c r="M231" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N231" s="14" t="str"/>
       <x:c r="O231" s="14" t="str"/>
@@ -10394,7 +10394,7 @@
         <x:v>wikipedia_verified</x:v>
       </x:c>
       <x:c r="L234" s="14" t="str">
-        <x:v>1987-1999 [not_established]; 2000-2011 [not_established]; 2012-2026 三沙市</x:v>
+        <x:v>1987-2011 [not_established]; 2012-2026 三沙市</x:v>
       </x:c>
       <x:c r="M234" s="15" t="str">
         <x:v>1</x:v>
@@ -14350,7 +14350,7 @@
         <x:v>wikipedia_verified</x:v>
       </x:c>
       <x:c r="L326" s="14" t="str">
-        <x:v>1987-1999 [not_established]; 2000-2002 [not_established]; 2003-2026 中卫市</x:v>
+        <x:v>1987-2002 [not_established]; 2003-2026 中卫市</x:v>
       </x:c>
       <x:c r="M326" s="15" t="str">
         <x:v>1</x:v>
@@ -15123,7 +15123,7 @@
         <x:v>1970</x:v>
       </x:c>
       <x:c r="I344" s="12" t="str">
-        <x:v>1993</x:v>
+        <x:v>1992</x:v>
       </x:c>
       <x:c r="J344" s="2" t="str">
         <x:v>abolished</x:v>
@@ -15132,7 +15132,7 @@
         <x:v>reviewed</x:v>
       </x:c>
       <x:c r="L344" s="14" t="str">
-        <x:v>1970-1993 雁北地区</x:v>
+        <x:v>1970-1992 雁北地区</x:v>
       </x:c>
       <x:c r="M344" s="15" t="str">
         <x:v>1</x:v>
@@ -15238,10 +15238,104 @@
         <x:v>https://zh.wikipedia.org/wiki/黔江地区</x:v>
       </x:c>
     </x:row>
+    <x:row r="347" ht="20" customHeight="1">
+      <x:c r="A347" s="2" t="str">
+        <x:v>CNUR-000346</x:v>
+      </x:c>
+      <x:c r="B347" s="2" t="str">
+        <x:v>HIST-GX-NANNING</x:v>
+      </x:c>
+      <x:c r="C347" s="2" t="str">
+        <x:v>南宁地区</x:v>
+      </x:c>
+      <x:c r="D347" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E347" s="2" t="str">
+        <x:v>广西壮族自治区</x:v>
+      </x:c>
+      <x:c r="F347" s="2" t="str">
+        <x:v>广西</x:v>
+      </x:c>
+      <x:c r="G347" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H347" s="2" t="str">
+        <x:v>1971</x:v>
+      </x:c>
+      <x:c r="I347" s="2" t="str">
+        <x:v>2001</x:v>
+      </x:c>
+      <x:c r="J347" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K347" s="2" t="str">
+        <x:v>reviewed_county_composition</x:v>
+      </x:c>
+      <x:c r="L347" s="2" t="str">
+        <x:v>1971-2001 南宁地区</x:v>
+      </x:c>
+      <x:c r="M347" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N347" s="2" t="str">
+        <x:v>撤销后主要分为崇左市并将五县划归南宁市</x:v>
+      </x:c>
+      <x:c r="O347" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/南宁地区</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348" ht="20" customHeight="1">
+      <x:c r="A348" s="2" t="str">
+        <x:v>CNUR-000347</x:v>
+      </x:c>
+      <x:c r="B348" s="2" t="str">
+        <x:v>HIST-GD-HUIYANG</x:v>
+      </x:c>
+      <x:c r="C348" s="2" t="str">
+        <x:v>惠阳地区</x:v>
+      </x:c>
+      <x:c r="D348" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E348" s="2" t="str">
+        <x:v>广东省</x:v>
+      </x:c>
+      <x:c r="F348" s="2" t="str">
+        <x:v>广东</x:v>
+      </x:c>
+      <x:c r="G348" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H348" s="2" t="str">
+        <x:v>1970</x:v>
+      </x:c>
+      <x:c r="I348" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="J348" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K348" s="2" t="str">
+        <x:v>reviewed_county_composition</x:v>
+      </x:c>
+      <x:c r="L348" s="2" t="str">
+        <x:v>1970-1987 惠阳地区</x:v>
+      </x:c>
+      <x:c r="M348" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N348" s="2" t="str">
+        <x:v>撤销后主要形成惠州市、汕尾市和河源市</x:v>
+      </x:c>
+      <x:c r="O348" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/惠阳地区</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdba77a3c4a34037"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01aebbe0ea2a43fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete prefecture lineage and level audit
</commit_message>
<xml_diff>
--- a/data/releases/v2.0/china_city_entity_master_V2.0.xlsx
+++ b/data/releases/v2.0/china_city_entity_master_V2.0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市总表" sheetId="1" r:id="R72f66fb9520143c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市总表" sheetId="1" r:id="R8e85c665558844e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -507,7 +507,7 @@
         <x:v>1987-2026 石家庄市</x:v>
       </x:c>
       <x:c r="M4" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str"/>
       <x:c r="O4" s="14" t="str"/>
@@ -4893,7 +4893,7 @@
         <x:v>1987-2026 安庆市</x:v>
       </x:c>
       <x:c r="M106" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N106" s="14" t="str"/>
       <x:c r="O106" s="14" t="str"/>
@@ -6598,7 +6598,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H146" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1989</x:v>
       </x:c>
       <x:c r="I146" s="12" t="str">
         <x:v>2026</x:v>
@@ -6610,7 +6610,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L146" s="14" t="str">
-        <x:v>1987-2026 日照市</x:v>
+        <x:v>1987-1988 [not_established]; 1989-2026 日照市</x:v>
       </x:c>
       <x:c r="M146" s="15" t="str">
         <x:v>0</x:v>
@@ -7731,7 +7731,7 @@
         <x:v>1987-2026 十堰市</x:v>
       </x:c>
       <x:c r="M172" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N172" s="14" t="str"/>
       <x:c r="O172" s="14" t="str"/>
@@ -7774,7 +7774,7 @@
         <x:v>1987-2026 宜昌市</x:v>
       </x:c>
       <x:c r="M173" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N173" s="14" t="str"/>
       <x:c r="O173" s="14" t="str"/>
@@ -7974,7 +7974,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H178" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1994</x:v>
       </x:c>
       <x:c r="I178" s="12" t="str">
         <x:v>2026</x:v>
@@ -7986,10 +7986,10 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L178" s="14" t="str">
-        <x:v>1987-1993 荆州地区; 1994-1995 荆沙市; 1996-2026 荆州市</x:v>
+        <x:v>1987-1993 [not_established]; 1994-1995 荆沙市; 1996-2026 荆州市</x:v>
       </x:c>
       <x:c r="M178" s="15" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N178" s="14" t="str"/>
       <x:c r="O178" s="14" t="str"/>
@@ -8490,7 +8490,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H190" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1988</x:v>
       </x:c>
       <x:c r="I190" s="12" t="str">
         <x:v>2026</x:v>
@@ -8502,7 +8502,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L190" s="14" t="str">
-        <x:v>1987-1993 大庸市; 1994-2026 张家界市</x:v>
+        <x:v>1987-1987 [not_established]; 1988-1993 大庸市; 1994-2026 张家界市</x:v>
       </x:c>
       <x:c r="M190" s="15" t="str">
         <x:v>1</x:v>
@@ -9479,7 +9479,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H213" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1988</x:v>
       </x:c>
       <x:c r="I213" s="12" t="str">
         <x:v>2026</x:v>
@@ -9491,7 +9491,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L213" s="14" t="str">
-        <x:v>1987-2026 东莞市</x:v>
+        <x:v>1987-1987 [not_established]; 1988-2026 东莞市</x:v>
       </x:c>
       <x:c r="M213" s="15" t="str">
         <x:v>0</x:v>
@@ -9522,7 +9522,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H214" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1988</x:v>
       </x:c>
       <x:c r="I214" s="12" t="str">
         <x:v>2026</x:v>
@@ -9534,7 +9534,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L214" s="14" t="str">
-        <x:v>1987-2026 中山市</x:v>
+        <x:v>1987-1987 [not_established]; 1988-2026 中山市</x:v>
       </x:c>
       <x:c r="M214" s="15" t="str">
         <x:v>0</x:v>
@@ -9565,7 +9565,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H215" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1991</x:v>
       </x:c>
       <x:c r="I215" s="12" t="str">
         <x:v>2026</x:v>
@@ -9577,7 +9577,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L215" s="14" t="str">
-        <x:v>1987-2026 潮州市</x:v>
+        <x:v>1987-1990 [not_established]; 1991-2026 潮州市</x:v>
       </x:c>
       <x:c r="M215" s="15" t="str">
         <x:v>0</x:v>
@@ -9608,7 +9608,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H216" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1991</x:v>
       </x:c>
       <x:c r="I216" s="12" t="str">
         <x:v>2026</x:v>
@@ -9620,7 +9620,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L216" s="14" t="str">
-        <x:v>1987-2026 揭阳市</x:v>
+        <x:v>1987-1990 [not_established]; 1991-2026 揭阳市</x:v>
       </x:c>
       <x:c r="M216" s="15" t="str">
         <x:v>0</x:v>
@@ -9651,7 +9651,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H217" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1994</x:v>
       </x:c>
       <x:c r="I217" s="12" t="str">
         <x:v>2026</x:v>
@@ -9663,7 +9663,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L217" s="14" t="str">
-        <x:v>1987-2026 云浮市</x:v>
+        <x:v>1987-1993 [not_established]; 1994-2026 云浮市</x:v>
       </x:c>
       <x:c r="M217" s="15" t="str">
         <x:v>0</x:v>
@@ -9995,7 +9995,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H225" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1995</x:v>
       </x:c>
       <x:c r="I225" s="12" t="str">
         <x:v>2026</x:v>
@@ -10007,7 +10007,7 @@
         <x:v>wikipedia_entity_verified</x:v>
       </x:c>
       <x:c r="L225" s="14" t="str">
-        <x:v>1987-2026 贵港市</x:v>
+        <x:v>1987-1994 [not_established]; 1995-2026 贵港市</x:v>
       </x:c>
       <x:c r="M225" s="15" t="str">
         <x:v>0</x:v>
@@ -10124,7 +10124,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H228" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>1997</x:v>
       </x:c>
       <x:c r="I228" s="12" t="str">
         <x:v>2026</x:v>
@@ -10136,10 +10136,10 @@
         <x:v>event_crosschecked</x:v>
       </x:c>
       <x:c r="L228" s="14" t="str">
-        <x:v>1987-1996 梧州地区; 1997-2001 贺州地区; 2002-2026 贺州市</x:v>
+        <x:v>1987-1996 [not_established]; 1997-2001 贺州地区; 2002-2026 贺州市</x:v>
       </x:c>
       <x:c r="M228" s="15" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N228" s="14" t="str"/>
       <x:c r="O228" s="14" t="str"/>
@@ -10210,7 +10210,7 @@
         <x:v>prefecture_research_entity</x:v>
       </x:c>
       <x:c r="H230" s="12" t="str">
-        <x:v>1987</x:v>
+        <x:v>2002</x:v>
       </x:c>
       <x:c r="I230" s="12" t="str">
         <x:v>2026</x:v>
@@ -10222,10 +10222,10 @@
         <x:v>event_crosschecked</x:v>
       </x:c>
       <x:c r="L230" s="14" t="str">
-        <x:v>1987-2001 柳州地区; 2002-2026 来宾市</x:v>
+        <x:v>1987-2001 [not_established]; 2002-2026 来宾市</x:v>
       </x:c>
       <x:c r="M230" s="15" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N230" s="14" t="str"/>
       <x:c r="O230" s="14" t="str"/>
@@ -15332,10 +15332,762 @@
         <x:v>https://zh.wikipedia.org/wiki/惠阳地区</x:v>
       </x:c>
     </x:row>
+    <x:row r="349" ht="20" customHeight="1">
+      <x:c r="A349" s="2" t="str">
+        <x:v>CNUR-000348</x:v>
+      </x:c>
+      <x:c r="B349" s="2" t="str">
+        <x:v>HIST-AH-ANQING</x:v>
+      </x:c>
+      <x:c r="C349" s="2" t="str">
+        <x:v>安庆地区</x:v>
+      </x:c>
+      <x:c r="D349" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E349" s="2" t="str">
+        <x:v>安徽省</x:v>
+      </x:c>
+      <x:c r="F349" s="2" t="str">
+        <x:v>安徽</x:v>
+      </x:c>
+      <x:c r="G349" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H349" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I349" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="J349" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K349" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L349" s="2" t="str">
+        <x:v>1987-1987 安庆地区</x:v>
+      </x:c>
+      <x:c r="M349" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N349" s="2" t="str">
+        <x:v>与既有安庆市合并并析设池州地区</x:v>
+      </x:c>
+      <x:c r="O349" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1988年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350" ht="20" customHeight="1">
+      <x:c r="A350" s="2" t="str">
+        <x:v>CNUR-000349</x:v>
+      </x:c>
+      <x:c r="B350" s="2" t="str">
+        <x:v>HIST-HB-YICHANG</x:v>
+      </x:c>
+      <x:c r="C350" s="2" t="str">
+        <x:v>宜昌地区</x:v>
+      </x:c>
+      <x:c r="D350" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E350" s="2" t="str">
+        <x:v>湖北省</x:v>
+      </x:c>
+      <x:c r="F350" s="2" t="str">
+        <x:v>湖北</x:v>
+      </x:c>
+      <x:c r="G350" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H350" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I350" s="2" t="str">
+        <x:v>1991</x:v>
+      </x:c>
+      <x:c r="J350" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K350" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L350" s="2" t="str">
+        <x:v>1987-1991 宜昌地区</x:v>
+      </x:c>
+      <x:c r="M350" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N350" s="2" t="str">
+        <x:v>撤销后整体并入既有宜昌市</x:v>
+      </x:c>
+      <x:c r="O350" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1992年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351" ht="20" customHeight="1">
+      <x:c r="A351" s="2" t="str">
+        <x:v>CNUR-000350</x:v>
+      </x:c>
+      <x:c r="B351" s="2" t="str">
+        <x:v>HIST-HE-SHIJIAZHUANG</x:v>
+      </x:c>
+      <x:c r="C351" s="2" t="str">
+        <x:v>石家庄地区</x:v>
+      </x:c>
+      <x:c r="D351" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E351" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F351" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G351" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H351" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I351" s="2" t="str">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="J351" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K351" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L351" s="2" t="str">
+        <x:v>1987-1992 石家庄地区</x:v>
+      </x:c>
+      <x:c r="M351" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N351" s="2" t="str">
+        <x:v>与既有石家庄市实行地市合并</x:v>
+      </x:c>
+      <x:c r="O351" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1993年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352" ht="20" customHeight="1">
+      <x:c r="A352" s="2" t="str">
+        <x:v>CNUR-000351</x:v>
+      </x:c>
+      <x:c r="B352" s="2" t="str">
+        <x:v>HIST-HE-ZHANGJIAKOU</x:v>
+      </x:c>
+      <x:c r="C352" s="2" t="str">
+        <x:v>张家口地区</x:v>
+      </x:c>
+      <x:c r="D352" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E352" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F352" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G352" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H352" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I352" s="2" t="str">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="J352" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K352" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L352" s="2" t="str">
+        <x:v>1987-1992 张家口地区</x:v>
+      </x:c>
+      <x:c r="M352" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N352" s="2" t="str">
+        <x:v>与既有张家口市实行地市合并</x:v>
+      </x:c>
+      <x:c r="O352" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1993年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353" ht="20" customHeight="1">
+      <x:c r="A353" s="2" t="str">
+        <x:v>CNUR-000352</x:v>
+      </x:c>
+      <x:c r="B353" s="2" t="str">
+        <x:v>HIST-HE-CANGZHOU</x:v>
+      </x:c>
+      <x:c r="C353" s="2" t="str">
+        <x:v>沧州地区</x:v>
+      </x:c>
+      <x:c r="D353" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E353" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F353" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G353" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H353" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I353" s="2" t="str">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="J353" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K353" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L353" s="2" t="str">
+        <x:v>1987-1992 沧州地区</x:v>
+      </x:c>
+      <x:c r="M353" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N353" s="2" t="str">
+        <x:v>与既有沧州市实行地市合并</x:v>
+      </x:c>
+      <x:c r="O353" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1993年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354" ht="20" customHeight="1">
+      <x:c r="A354" s="2" t="str">
+        <x:v>CNUR-000353</x:v>
+      </x:c>
+      <x:c r="B354" s="2" t="str">
+        <x:v>HIST-HE-HANDAN</x:v>
+      </x:c>
+      <x:c r="C354" s="2" t="str">
+        <x:v>邯郸地区</x:v>
+      </x:c>
+      <x:c r="D354" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E354" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F354" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G354" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H354" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I354" s="2" t="str">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="J354" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K354" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L354" s="2" t="str">
+        <x:v>1987-1992 邯郸地区</x:v>
+      </x:c>
+      <x:c r="M354" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N354" s="2" t="str">
+        <x:v>与既有邯郸市实行地市合并</x:v>
+      </x:c>
+      <x:c r="O354" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1993年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355" ht="20" customHeight="1">
+      <x:c r="A355" s="2" t="str">
+        <x:v>CNUR-000354</x:v>
+      </x:c>
+      <x:c r="B355" s="2" t="str">
+        <x:v>HIST-HE-XINGTAI</x:v>
+      </x:c>
+      <x:c r="C355" s="2" t="str">
+        <x:v>邢台地区</x:v>
+      </x:c>
+      <x:c r="D355" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E355" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F355" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G355" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H355" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I355" s="2" t="str">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="J355" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K355" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L355" s="2" t="str">
+        <x:v>1987-1992 邢台地区</x:v>
+      </x:c>
+      <x:c r="M355" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N355" s="2" t="str">
+        <x:v>与既有邢台市实行地市合并</x:v>
+      </x:c>
+      <x:c r="O355" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1993年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356" ht="20" customHeight="1">
+      <x:c r="A356" s="2" t="str">
+        <x:v>CNUR-000355</x:v>
+      </x:c>
+      <x:c r="B356" s="2" t="str">
+        <x:v>HIST-HE-CHENGDE</x:v>
+      </x:c>
+      <x:c r="C356" s="2" t="str">
+        <x:v>承德地区</x:v>
+      </x:c>
+      <x:c r="D356" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E356" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F356" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G356" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H356" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I356" s="2" t="str">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="J356" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K356" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L356" s="2" t="str">
+        <x:v>1987-1992 承德地区</x:v>
+      </x:c>
+      <x:c r="M356" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N356" s="2" t="str">
+        <x:v>与既有承德市实行地市合并</x:v>
+      </x:c>
+      <x:c r="O356" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1993年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357" ht="20" customHeight="1">
+      <x:c r="A357" s="2" t="str">
+        <x:v>CNUR-000356</x:v>
+      </x:c>
+      <x:c r="B357" s="2" t="str">
+        <x:v>HIST-HE-BAODING</x:v>
+      </x:c>
+      <x:c r="C357" s="2" t="str">
+        <x:v>保定地区</x:v>
+      </x:c>
+      <x:c r="D357" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E357" s="2" t="str">
+        <x:v>河北省</x:v>
+      </x:c>
+      <x:c r="F357" s="2" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="G357" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H357" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I357" s="2" t="str">
+        <x:v>1993</x:v>
+      </x:c>
+      <x:c r="J357" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K357" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L357" s="2" t="str">
+        <x:v>1987-1993 保定地区</x:v>
+      </x:c>
+      <x:c r="M357" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N357" s="2" t="str">
+        <x:v>与既有保定市合并组建新的保定市</x:v>
+      </x:c>
+      <x:c r="O357" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1994年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358" ht="20" customHeight="1">
+      <x:c r="A358" s="2" t="str">
+        <x:v>CNUR-000357</x:v>
+      </x:c>
+      <x:c r="B358" s="2" t="str">
+        <x:v>HIST-HB-YUNYANG</x:v>
+      </x:c>
+      <x:c r="C358" s="2" t="str">
+        <x:v>郧阳地区</x:v>
+      </x:c>
+      <x:c r="D358" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E358" s="2" t="str">
+        <x:v>湖北省</x:v>
+      </x:c>
+      <x:c r="F358" s="2" t="str">
+        <x:v>湖北</x:v>
+      </x:c>
+      <x:c r="G358" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H358" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I358" s="2" t="str">
+        <x:v>1993</x:v>
+      </x:c>
+      <x:c r="J358" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K358" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L358" s="2" t="str">
+        <x:v>1987-1993 郧阳地区</x:v>
+      </x:c>
+      <x:c r="M358" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N358" s="2" t="str">
+        <x:v>撤销后与既有十堰市合并</x:v>
+      </x:c>
+      <x:c r="O358" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1994年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359" ht="20" customHeight="1">
+      <x:c r="A359" s="2" t="str">
+        <x:v>CNUR-000358</x:v>
+      </x:c>
+      <x:c r="B359" s="2" t="str">
+        <x:v>HIST-HB-JINGZHOU</x:v>
+      </x:c>
+      <x:c r="C359" s="2" t="str">
+        <x:v>荆州地区</x:v>
+      </x:c>
+      <x:c r="D359" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E359" s="2" t="str">
+        <x:v>湖北省</x:v>
+      </x:c>
+      <x:c r="F359" s="2" t="str">
+        <x:v>湖北</x:v>
+      </x:c>
+      <x:c r="G359" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H359" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I359" s="2" t="str">
+        <x:v>1993</x:v>
+      </x:c>
+      <x:c r="J359" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K359" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L359" s="2" t="str">
+        <x:v>1987-1993 荆州地区</x:v>
+      </x:c>
+      <x:c r="M359" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N359" s="2" t="str">
+        <x:v>与原地级沙市市共同组建荆沙市</x:v>
+      </x:c>
+      <x:c r="O359" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1994年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360" ht="20" customHeight="1">
+      <x:c r="A360" s="2" t="str">
+        <x:v>CNUR-000359</x:v>
+      </x:c>
+      <x:c r="B360" s="2" t="str">
+        <x:v>HIST-HB-SHASHI</x:v>
+      </x:c>
+      <x:c r="C360" s="2" t="str">
+        <x:v>沙市市</x:v>
+      </x:c>
+      <x:c r="D360" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E360" s="2" t="str">
+        <x:v>湖北省</x:v>
+      </x:c>
+      <x:c r="F360" s="2" t="str">
+        <x:v>湖北</x:v>
+      </x:c>
+      <x:c r="G360" s="2" t="str">
+        <x:v>abolished_prefecture_level_city</x:v>
+      </x:c>
+      <x:c r="H360" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I360" s="2" t="str">
+        <x:v>1993</x:v>
+      </x:c>
+      <x:c r="J360" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K360" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L360" s="2" t="str">
+        <x:v>1987-1993 沙市市</x:v>
+      </x:c>
+      <x:c r="M360" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N360" s="2" t="str">
+        <x:v>与荆州地区共同组建荆沙市</x:v>
+      </x:c>
+      <x:c r="O360" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1994年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361" ht="20" customHeight="1">
+      <x:c r="A361" s="2" t="str">
+        <x:v>CNUR-000360</x:v>
+      </x:c>
+      <x:c r="B361" s="2" t="str">
+        <x:v>HIST-HLJ-SONGHUAJIANG</x:v>
+      </x:c>
+      <x:c r="C361" s="2" t="str">
+        <x:v>松花江地区</x:v>
+      </x:c>
+      <x:c r="D361" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E361" s="2" t="str">
+        <x:v>黑龙江省</x:v>
+      </x:c>
+      <x:c r="F361" s="2" t="str">
+        <x:v>黑龙江</x:v>
+      </x:c>
+      <x:c r="G361" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H361" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I361" s="2" t="str">
+        <x:v>1995</x:v>
+      </x:c>
+      <x:c r="J361" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K361" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L361" s="2" t="str">
+        <x:v>1987-1995 松花江地区</x:v>
+      </x:c>
+      <x:c r="M361" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N361" s="2" t="str">
+        <x:v>与既有哈尔滨市合并</x:v>
+      </x:c>
+      <x:c r="O361" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1996年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="20" customHeight="1">
+      <x:c r="A362" s="2" t="str">
+        <x:v>CNUR-000361</x:v>
+      </x:c>
+      <x:c r="B362" s="2" t="str">
+        <x:v>HIST-GX-GUILIN</x:v>
+      </x:c>
+      <x:c r="C362" s="2" t="str">
+        <x:v>桂林地区</x:v>
+      </x:c>
+      <x:c r="D362" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E362" s="2" t="str">
+        <x:v>广西壮族自治区</x:v>
+      </x:c>
+      <x:c r="F362" s="2" t="str">
+        <x:v>广西</x:v>
+      </x:c>
+      <x:c r="G362" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H362" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I362" s="2" t="str">
+        <x:v>1997</x:v>
+      </x:c>
+      <x:c r="J362" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K362" s="2" t="str">
+        <x:v>reviewed_event_row</x:v>
+      </x:c>
+      <x:c r="L362" s="2" t="str">
+        <x:v>1987-1997 桂林地区</x:v>
+      </x:c>
+      <x:c r="M362" s="2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N362" s="2" t="str">
+        <x:v>与既有桂林市合并</x:v>
+      </x:c>
+      <x:c r="O362" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1998年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363" ht="20" customHeight="1">
+      <x:c r="A363" s="2" t="str">
+        <x:v>CNUR-000362</x:v>
+      </x:c>
+      <x:c r="B363" s="2" t="str">
+        <x:v>HIST-GX-LIUZHOU</x:v>
+      </x:c>
+      <x:c r="C363" s="2" t="str">
+        <x:v>柳州地区</x:v>
+      </x:c>
+      <x:c r="D363" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E363" s="2" t="str">
+        <x:v>广西壮族自治区</x:v>
+      </x:c>
+      <x:c r="F363" s="2" t="str">
+        <x:v>广西</x:v>
+      </x:c>
+      <x:c r="G363" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H363" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I363" s="2" t="str">
+        <x:v>2001</x:v>
+      </x:c>
+      <x:c r="J363" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K363" s="2" t="str">
+        <x:v>reviewed_county_composition</x:v>
+      </x:c>
+      <x:c r="L363" s="2" t="str">
+        <x:v>1987-2001 柳州地区</x:v>
+      </x:c>
+      <x:c r="M363" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N363" s="2" t="str">
+        <x:v>撤销后主要分为来宾市并将四县划归柳州市</x:v>
+      </x:c>
+      <x:c r="O363" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/柳州地区</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="20" customHeight="1">
+      <x:c r="A364" s="2" t="str">
+        <x:v>CNUR-000363</x:v>
+      </x:c>
+      <x:c r="B364" s="2" t="str">
+        <x:v>HIST-GX-WUZHOU</x:v>
+      </x:c>
+      <x:c r="C364" s="2" t="str">
+        <x:v>梧州地区</x:v>
+      </x:c>
+      <x:c r="D364" s="2" t="str">
+        <x:v>historical_entity</x:v>
+      </x:c>
+      <x:c r="E364" s="2" t="str">
+        <x:v>广西壮族自治区</x:v>
+      </x:c>
+      <x:c r="F364" s="2" t="str">
+        <x:v>广西</x:v>
+      </x:c>
+      <x:c r="G364" s="2" t="str">
+        <x:v>abolished_prefecture</x:v>
+      </x:c>
+      <x:c r="H364" s="2" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="I364" s="2" t="str">
+        <x:v>1996</x:v>
+      </x:c>
+      <x:c r="J364" s="2" t="str">
+        <x:v>abolished</x:v>
+      </x:c>
+      <x:c r="K364" s="2" t="str">
+        <x:v>reviewed_county_composition</x:v>
+      </x:c>
+      <x:c r="L364" s="2" t="str">
+        <x:v>1987-1996 梧州地区</x:v>
+      </x:c>
+      <x:c r="M364" s="2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N364" s="2" t="str">
+        <x:v>更名贺州地区时四县留归贺州、三县市划归既有梧州市</x:v>
+      </x:c>
+      <x:c r="O364" s="2" t="str">
+        <x:v>https://zh.wikipedia.org/wiki/1997年中华人民共和国县级以上行政区划变更列表</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01aebbe0ea2a43fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c4f683714d4525"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>